<commit_message>
atualização dia 19 de de outubro
</commit_message>
<xml_diff>
--- a/dados/banco_dados.xlsx
+++ b/dados/banco_dados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="dicionario" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="produto" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="loja" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="oferta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dicionario" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="produto" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="loja" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="oferta" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -335,8 +335,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tb_oferta" displayName="tb_oferta" ref="A3:I246" headerRowCount="1">
-  <autoFilter ref="A3:I246"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tb_oferta" displayName="tb_oferta" ref="A3:I272" headerRowCount="1">
+  <autoFilter ref="A3:I272"/>
   <tableColumns count="9">
     <tableColumn id="1" name="id_oferta"/>
     <tableColumn id="2" name="id_produto"/>
@@ -661,7 +661,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Modelo estrela do pipeline de preços · atualizado em 18/10/2026 13:05</t>
+          <t>Modelo estrela do pipeline de preços · atualizado em 19/10/2026 11:07</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I246"/>
+  <dimension ref="A1:I272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9751,6 +9751,864 @@
       </c>
       <c r="I246" s="31" t="n">
         <v>46313.54508101852</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="24" t="n">
+        <v>244</v>
+      </c>
+      <c r="B247" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C247" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D247" s="32" t="n">
+        <v>1199.99</v>
+      </c>
+      <c r="E247" s="32" t="n">
+        <v>1134.33</v>
+      </c>
+      <c r="F247" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G247" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H247" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/320797/processador-amd-ryzen-7-5700x-3-4ghz-4-6ghz-max-turbo-cache-36mb-8-nucleos-16-threads-am4-sem-video-integrado-100-100000926wof</t>
+        </is>
+      </c>
+      <c r="I247" s="34" t="n">
+        <v>46314.12506944445</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="22" t="n">
+        <v>245</v>
+      </c>
+      <c r="B248" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C248" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D248" s="29" t="n">
+        <v>1549.99</v>
+      </c>
+      <c r="E248" s="29" t="n">
+        <v>1054.54</v>
+      </c>
+      <c r="F248" s="30" t="b">
+        <v>1</v>
+      </c>
+      <c r="G248" s="23" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="H248" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/405799/processador-amd-ryzen-5-7600-3-8ghz-5-1ghz-max-turbo-cache-38mb-6-nucleos-12-threads-am5-com-video-integrado-100-100001015box</t>
+        </is>
+      </c>
+      <c r="I248" s="31" t="n">
+        <v>46314.12511574074</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="24" t="n">
+        <v>246</v>
+      </c>
+      <c r="B249" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C249" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D249" s="32" t="n">
+        <v>1978.9</v>
+      </c>
+      <c r="E249" s="32" t="n">
+        <v>1962.47</v>
+      </c>
+      <c r="F249" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G249" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H249" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/466557/processador-amd-ryzen-7-7800x3d-4-2ghz-5-0ghz-max-turbo-cache-104mb-am5-c-video-e-sem-cooler-100-100000910wof</t>
+        </is>
+      </c>
+      <c r="I249" s="34" t="n">
+        <v>46314.12515046296</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="22" t="n">
+        <v>247</v>
+      </c>
+      <c r="B250" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C250" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D250" s="29" t="n">
+        <v>859.99</v>
+      </c>
+      <c r="E250" s="29" t="n">
+        <v>973.4400000000001</v>
+      </c>
+      <c r="F250" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G250" s="23" t="inlineStr">
+        <is>
+          <t>Boa compra</t>
+        </is>
+      </c>
+      <c r="H250" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/283718/processador-intel-core-i5-12400f-2-5ghz-4-4ghz-max-turbo-cache-18mb-6-nucleos-12-threads-lga-1700-sem-video-integrado-bx8071512400f</t>
+        </is>
+      </c>
+      <c r="I250" s="31" t="n">
+        <v>46314.12518518518</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="24" t="n">
+        <v>248</v>
+      </c>
+      <c r="B251" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C251" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D251" s="32" t="n">
+        <v>1069.99</v>
+      </c>
+      <c r="E251" s="32" t="n">
+        <v>1036.36</v>
+      </c>
+      <c r="F251" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G251" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H251" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/531209/processador-intel-core-i5-14400f-14-geracao-3-5-ghz-4-7-ghz-turbo-cache-20mb-10-nucleos-16-threads-lga1700-sem-video-integrado-bx8071514400f</t>
+        </is>
+      </c>
+      <c r="I251" s="34" t="n">
+        <v>46314.12520833333</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="22" t="n">
+        <v>249</v>
+      </c>
+      <c r="B252" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="C252" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D252" s="29" t="n">
+        <v>2899.9</v>
+      </c>
+      <c r="E252" s="29" t="n">
+        <v>2802.28</v>
+      </c>
+      <c r="F252" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G252" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H252" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/903752/gpu-inno3d-geforce-rtx-5060-twin-x2-8gb-128bits-gddr7-n50602-08d7-195071n</t>
+        </is>
+      </c>
+      <c r="I252" s="31" t="n">
+        <v>46314.12524305555</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="24" t="n">
+        <v>250</v>
+      </c>
+      <c r="B253" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C253" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D253" s="32" t="n">
+        <v>5499.99</v>
+      </c>
+      <c r="E253" s="32" t="n">
+        <v>5489.09</v>
+      </c>
+      <c r="F253" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G253" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H253" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/989623/placa-de-video-palit-rtx-5070-infinity-3-nvidia-geforce-12gb-gddr7-192bit-3-dp-e-hdmi-ne75070019k9-gb2050s</t>
+        </is>
+      </c>
+      <c r="I253" s="34" t="n">
+        <v>46314.1252662037</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="22" t="n">
+        <v>251</v>
+      </c>
+      <c r="B254" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="C254" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D254" s="29" t="n">
+        <v>2199.99</v>
+      </c>
+      <c r="E254" s="29" t="n">
+        <v>2336.32</v>
+      </c>
+      <c r="F254" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G254" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H254" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/996572/placa-de-video-husky-alpha-rtx-3060-nvidia-12gb-gddr6-192-bit-dual-fan-hdmi-3x-displayport-hvg023060</t>
+        </is>
+      </c>
+      <c r="I254" s="31" t="n">
+        <v>46314.1253125</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="24" t="n">
+        <v>252</v>
+      </c>
+      <c r="B255" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="C255" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D255" s="32" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="E255" s="32" t="n">
+        <v>1951.04</v>
+      </c>
+      <c r="F255" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G255" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H255" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/459144/placa-de-video-rx-7600-challenger-asrock-amd-radeon-8gb-gddr6-90-ga41zz-00uanf</t>
+        </is>
+      </c>
+      <c r="I255" s="34" t="n">
+        <v>46314.12533564815</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="22" t="n">
+        <v>253</v>
+      </c>
+      <c r="B256" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="C256" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D256" s="29" t="n">
+        <v>519.99</v>
+      </c>
+      <c r="E256" s="29" t="n">
+        <v>541.63</v>
+      </c>
+      <c r="F256" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G256" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H256" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/313833/memoria-kingston-fury-beast-8gb-3200mhz-ddr4-cl16-preto-kf432c16bb-8</t>
+        </is>
+      </c>
+      <c r="I256" s="31" t="n">
+        <v>46314.12537037037</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="24" t="n">
+        <v>254</v>
+      </c>
+      <c r="B257" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="C257" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D257" s="32" t="n">
+        <v>1016.41</v>
+      </c>
+      <c r="E257" s="32" t="n">
+        <v>1005.95</v>
+      </c>
+      <c r="F257" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G257" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H257" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/938663/memoria-ram-kingston-hyperx-ddr4-16gb-2666mhz-cl16-udimm-desktop</t>
+        </is>
+      </c>
+      <c r="I257" s="34" t="n">
+        <v>46314.12539351852</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="22" t="n">
+        <v>255</v>
+      </c>
+      <c r="B258" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="C258" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D258" s="29" t="n">
+        <v>2049.99</v>
+      </c>
+      <c r="E258" s="29" t="n">
+        <v>2119.18</v>
+      </c>
+      <c r="F258" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G258" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H258" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/285967/memoria-ram-kingston-fury-beast-16gb-5600mhz-ddr5-cl40-para-intel-xmp-preto-kf556c40bb-16</t>
+        </is>
+      </c>
+      <c r="I258" s="31" t="n">
+        <v>46314.12542824074</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="24" t="n">
+        <v>256</v>
+      </c>
+      <c r="B259" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="C259" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D259" s="32" t="n">
+        <v>1139.05</v>
+      </c>
+      <c r="E259" s="32" t="n">
+        <v>1063.82</v>
+      </c>
+      <c r="F259" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G259" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H259" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/1021928/ssd-kingston-nv3-1tb-m-2-2280-nvme-gen4-desempenho-e-eficiencia-para-upgrade-de-pc-snv3s-1000g</t>
+        </is>
+      </c>
+      <c r="I259" s="34" t="n">
+        <v>46314.12545138889</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="22" t="n">
+        <v>257</v>
+      </c>
+      <c r="B260" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="C260" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D260" s="29" t="n">
+        <v>2399</v>
+      </c>
+      <c r="E260" s="29" t="n">
+        <v>2085.19</v>
+      </c>
+      <c r="F260" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G260" s="23" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="H260" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/464267/ssd-samsung-990-pro-1tb-nvme-m-2-2280-mz-v9p1t0b-am-</t>
+        </is>
+      </c>
+      <c r="I260" s="31" t="n">
+        <v>46314.12547453704</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="24" t="n">
+        <v>258</v>
+      </c>
+      <c r="B261" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="C261" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D261" s="32" t="n">
+        <v>476.99</v>
+      </c>
+      <c r="E261" s="32" t="n">
+        <v>535.87</v>
+      </c>
+      <c r="F261" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G261" s="25" t="inlineStr">
+        <is>
+          <t>Boa compra</t>
+        </is>
+      </c>
+      <c r="H261" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/781777/ssd-kingston-a400-480gb-sata-iii-2-5-leitura-500mb-s-gravacao-450mb-s-preto-sa400s37-480g</t>
+        </is>
+      </c>
+      <c r="I261" s="34" t="n">
+        <v>46314.12550925926</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="22" t="n">
+        <v>259</v>
+      </c>
+      <c r="B262" s="22" t="n">
+        <v>17</v>
+      </c>
+      <c r="C262" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D262" s="29" t="n">
+        <v>759</v>
+      </c>
+      <c r="E262" s="29" t="n">
+        <v>761.6799999999999</v>
+      </c>
+      <c r="F262" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G262" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H262" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/172706/placa-mae-asus-tuf-gaming-b550m-plus-amd-am4-matx-ddr4-m-2-aura-para-fita-rgb-90mb14a0-c1bay0</t>
+        </is>
+      </c>
+      <c r="I262" s="31" t="n">
+        <v>46314.12553240741</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="24" t="n">
+        <v>260</v>
+      </c>
+      <c r="B263" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="C263" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D263" s="32" t="n">
+        <v>896.99</v>
+      </c>
+      <c r="E263" s="32" t="n">
+        <v>971.5700000000001</v>
+      </c>
+      <c r="F263" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G263" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H263" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/524346/placa-mae-msi-pro-b650m-p-amd-am5-m-atx-ddr5-pro-b650m-p</t>
+        </is>
+      </c>
+      <c r="I263" s="34" t="n">
+        <v>46314.12556712963</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="22" t="n">
+        <v>261</v>
+      </c>
+      <c r="B264" s="22" t="n">
+        <v>19</v>
+      </c>
+      <c r="C264" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D264" s="29" t="n">
+        <v>359.99</v>
+      </c>
+      <c r="E264" s="29" t="n">
+        <v>364.99</v>
+      </c>
+      <c r="F264" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G264" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H264" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/516056/fonte-corsair-cx-series-cx650-650w-80-plus-bronze-com-cabo-preto-cp-9020278-br</t>
+        </is>
+      </c>
+      <c r="I264" s="31" t="n">
+        <v>46314.12560185185</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="24" t="n">
+        <v>262</v>
+      </c>
+      <c r="B265" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="C265" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D265" s="32" t="n">
+        <v>349.99</v>
+      </c>
+      <c r="E265" s="32" t="n">
+        <v>296.98</v>
+      </c>
+      <c r="F265" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G265" s="25" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="H265" s="27" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/369658/fonte-msi-mag-a650bn-650w-80-plus-bronze-pfc-ativo-com-cabo-preto-306-7zp2b22-ce0</t>
+        </is>
+      </c>
+      <c r="I265" s="34" t="n">
+        <v>46314.125625</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="22" t="n">
+        <v>263</v>
+      </c>
+      <c r="B266" s="22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C266" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D266" s="29" t="n">
+        <v>699.89</v>
+      </c>
+      <c r="E266" s="29" t="n">
+        <v>708.9</v>
+      </c>
+      <c r="F266" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G266" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H266" s="26" t="inlineStr">
+        <is>
+          <t>https://www.kabum.com.br/produto/514895/fonte-xpg-core-reactor-ii-ve-750w-80-plus-gold-modular-pfc-ativo-preto-75261425</t>
+        </is>
+      </c>
+      <c r="I266" s="31" t="n">
+        <v>46314.12564814815</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="24" t="n">
+        <v>264</v>
+      </c>
+      <c r="B267" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C267" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D267" s="32" t="n">
+        <v>1199.99</v>
+      </c>
+      <c r="E267" s="32" t="n">
+        <v>1134.33</v>
+      </c>
+      <c r="F267" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G267" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H267" s="27" t="inlineStr">
+        <is>
+          <t>https://www.pichau.com.br/processador-amd-ryzen-7-5700x-8-core-16-threads-3-4ghz-4-6ghz-turbo-cache-36mb-am4-100-100000926wof</t>
+        </is>
+      </c>
+      <c r="I267" s="34" t="n">
+        <v>46314.12577546296</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="22" t="n">
+        <v>265</v>
+      </c>
+      <c r="B268" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C268" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D268" s="29" t="n">
+        <v>1999.99</v>
+      </c>
+      <c r="E268" s="29" t="n">
+        <v>1962.47</v>
+      </c>
+      <c r="F268" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G268" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H268" s="26" t="inlineStr">
+        <is>
+          <t>https://www.pichau.com.br/processador-amd-ryzen-7-7800x3d-8-core-16-threads-4-2ghz-5-0ghzturbo-cache-104mb-am5-100-100000910wof</t>
+        </is>
+      </c>
+      <c r="I268" s="31" t="n">
+        <v>46314.12577546296</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="24" t="n">
+        <v>266</v>
+      </c>
+      <c r="B269" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="C269" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D269" s="32" t="n">
+        <v>1199.9</v>
+      </c>
+      <c r="E269" s="32" t="n">
+        <v>1063.82</v>
+      </c>
+      <c r="F269" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G269" s="25" t="inlineStr">
+        <is>
+          <t>Evitar</t>
+        </is>
+      </c>
+      <c r="H269" s="27" t="inlineStr">
+        <is>
+          <t>https://www.terabyteshop.com.br/produto/31564/ssd-kingston-nv3-1tb-m2-nvme-2280-pcie-40-leitura-6000mbs-e-gravacao-4000mbs-snv3s1000g</t>
+        </is>
+      </c>
+      <c r="I269" s="34" t="n">
+        <v>46314.12585648148</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="22" t="n">
+        <v>267</v>
+      </c>
+      <c r="B270" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="C270" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D270" s="29" t="n">
+        <v>569.9</v>
+      </c>
+      <c r="E270" s="29" t="n">
+        <v>535.87</v>
+      </c>
+      <c r="F270" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G270" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H270" s="26" t="inlineStr">
+        <is>
+          <t>https://www.terabyteshop.com.br/produto/19382/ssd-kingston-a400-480gb-sata-iii-leitura-500mbs-gravacao-450mbs-sa400s37480g-imp</t>
+        </is>
+      </c>
+      <c r="I270" s="31" t="n">
+        <v>46314.12585648148</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="24" t="n">
+        <v>268</v>
+      </c>
+      <c r="B271" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="C271" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D271" s="32" t="n">
+        <v>1959.99</v>
+      </c>
+      <c r="E271" s="32" t="n">
+        <v>1951.04</v>
+      </c>
+      <c r="F271" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G271" s="25" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H271" s="27" t="inlineStr">
+        <is>
+          <t>https://www.pichau.com.br/placa-de-video-powercolor-radeon-rx-7600-fighter-8gb-gddr6-128-bit-rx7600-8g-f-v2</t>
+        </is>
+      </c>
+      <c r="I271" s="34" t="n">
+        <v>46314.46310185185</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="22" t="n">
+        <v>269</v>
+      </c>
+      <c r="B272" s="22" t="n">
+        <v>17</v>
+      </c>
+      <c r="C272" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D272" s="29" t="n">
+        <v>779.99</v>
+      </c>
+      <c r="E272" s="29" t="n">
+        <v>761.6799999999999</v>
+      </c>
+      <c r="F272" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G272" s="23" t="inlineStr">
+        <is>
+          <t>Preço médio</t>
+        </is>
+      </c>
+      <c r="H272" s="26" t="inlineStr">
+        <is>
+          <t>https://www.terabyteshop.com.br/produto/13983/placa-mae-asus-tuf-gaming-b550m-plus-chipset-b550-amd-am4-matx-ddr4</t>
+        </is>
+      </c>
+      <c r="I272" s="31" t="n">
+        <v>46314.46341435185</v>
       </c>
     </row>
   </sheetData>
@@ -10001,10 +10859,36 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H244" r:id="rId241"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H245" r:id="rId242"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H246" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H247" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H248" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H249" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H250" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H251" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H252" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H253" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H254" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H255" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H256" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H257" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H258" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H259" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H260" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H261" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H262" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H263" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H264" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H265" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H266" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H267" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H268" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H269" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H270" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H271" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H272" r:id="rId269"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId244"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId270"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>